<commit_message>
Refactor data normalization and profile mapping to enhance data processing and maintainability
</commit_message>
<xml_diff>
--- a/data/input/Items Status.xlsx
+++ b/data/input/Items Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\IT\Projects\Crd Smart Grouping\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E9BFE4-46BB-428B-861F-0AB3AD1CAC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DE6B81-5D32-44F6-819E-0450E9AD1C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="3015" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33450" yWindow="4320" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3336,6 +3336,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M161"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="131.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="128.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="121.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="122" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>